<commit_message>
PRSO.OL CR:c|low|misclassified. + Excel + D&A
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/PRSO.OL.xlsx
+++ b/data/obx_xlsx/PRSO.OL.xlsx
@@ -2635,14 +2635,8 @@
       <c r="L26" s="16"/>
       <c r="M26" s="16"/>
       <c r="N26" s="16"/>
-      <c r="O26" s="15">
-        <v>770.46</v>
-      </c>
       <c r="P26" s="16"/>
       <c r="Q26" s="16"/>
-      <c r="R26" s="15">
-        <v>442.19</v>
-      </c>
       <c r="S26" s="16"/>
       <c r="T26" s="16"/>
       <c r="U26" s="16"/>
@@ -2692,7 +2686,9 @@
       <c r="N27" s="15">
         <v>690.63</v>
       </c>
-      <c r="O27" s="16"/>
+      <c r="O27" s="15">
+        <v>770.46</v>
+      </c>
       <c r="P27" s="15">
         <v>379.29</v>
       </c>
@@ -2700,7 +2696,7 @@
         <v>379.96</v>
       </c>
       <c r="R27" s="15">
-        <v>297.72</v>
+        <v>442.19</v>
       </c>
       <c r="S27" s="15">
         <v>708.04</v>
@@ -2764,7 +2760,9 @@
       </c>
       <c r="P28" s="16"/>
       <c r="Q28" s="16"/>
-      <c r="R28" s="16"/>
+      <c r="R28" s="15">
+        <v>297.72</v>
+      </c>
       <c r="S28" s="16"/>
       <c r="T28" s="16"/>
       <c r="U28" s="16"/>

</xml_diff>